<commit_message>
feat(data): generate master thesis bulk upload file containing 2 records for each of the 4 master programs
</commit_message>
<xml_diff>
--- a/backend/excel-templates/New-Test-data/master_msncs_test_data.xlsx
+++ b/backend/excel-templates/New-Test-data/master_msncs_test_data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,19 +442,19 @@
         <v>083</v>
       </c>
       <c r="E2" t="str">
-        <v>Cluster 1</v>
+        <v>Computer networks and security</v>
       </c>
       <c r="F2" t="str">
-        <v>MSc in Network and Cyber Security</v>
+        <v>MSNCS</v>
       </c>
       <c r="G2" t="str">
-        <v>Dr. Nilima Joshi</v>
+        <v>Prof. Dr. Dinesh Koirala</v>
       </c>
       <c r="H2" t="str">
         <v>Dr. Prajwal Ghimire</v>
       </c>
       <c r="I2" t="str">
-        <v>Dr. Bidur Khadka</v>
+        <v>Dr. Anisha Rana</v>
       </c>
     </row>
     <row r="3">
@@ -471,198 +471,24 @@
         <v>083</v>
       </c>
       <c r="E3" t="str">
-        <v>Cluster 1</v>
+        <v>Computer networks and security</v>
       </c>
       <c r="F3" t="str">
-        <v>MSc in Network and Cyber Security</v>
+        <v>MSNCS</v>
       </c>
       <c r="G3" t="str">
-        <v>Prof. Dr. Raju Poudel</v>
+        <v>Assoc. Prof. Dr. Meena Shrestha</v>
       </c>
       <c r="H3" t="str">
-        <v>Prof. Dr. Lokendra Dhakal</v>
+        <v>Dr. Bidur Khadka</v>
       </c>
       <c r="I3" t="str">
-        <v>Assoc. Prof. Dr. Manisha Aryal</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Oshan Kumal</v>
-      </c>
-      <c r="B4" t="str">
-        <v>083MSNCS03</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Secure E-Voting System Using Blockchain Technology</v>
-      </c>
-      <c r="D4" t="str">
-        <v>083</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Cluster 1</v>
-      </c>
-      <c r="F4" t="str">
-        <v>MSc in Network and Cyber Security</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Prof. Dr. Dinesh Koirala</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Dr. Anisha Rana</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Dr. Sabin Wagle</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Purnima Timalsina</v>
-      </c>
-      <c r="B5" t="str">
-        <v>083MSNCS04</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Phishing Detection Using Machine Learning on Email Headers</v>
-      </c>
-      <c r="D5" t="str">
-        <v>083</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Cluster 1</v>
-      </c>
-      <c r="F5" t="str">
-        <v>MSc in Network and Cyber Security</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Assoc. Prof. Dr. Meena Shrestha</v>
-      </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
-      <c r="I5" t="str">
-        <v>Dr. Prajwal Ghimire</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Rajan Dangol</v>
-      </c>
-      <c r="B6" t="str">
-        <v>083MSNCS05</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Implementation of SIEM for Small Enterprise Networks</v>
-      </c>
-      <c r="D6" t="str">
-        <v>083</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Cluster 1</v>
-      </c>
-      <c r="F6" t="str">
-        <v>MSc in Network and Cyber Security</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Dr. Kiran Adhikari</v>
-      </c>
-      <c r="H6" t="str">
-        <v>Assoc. Prof. Dr. Manisha Aryal</v>
-      </c>
-      <c r="I6" t="str">
-        <v>Prof. Dr. Lokendra Dhakal</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Sabita Acharya</v>
-      </c>
-      <c r="B7" t="str">
-        <v>083MSNCS06</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Zero Trust Network Architecture for Cloud Environments</v>
-      </c>
-      <c r="D7" t="str">
-        <v>083</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Cluster 1</v>
-      </c>
-      <c r="F7" t="str">
-        <v>MSc in Network and Cyber Security</v>
-      </c>
-      <c r="G7" t="str">
-        <v/>
-      </c>
-      <c r="H7" t="str">
-        <v>Dr. Sabin Wagle</v>
-      </c>
-      <c r="I7" t="str">
-        <v>Dr. Anisha Rana</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Tej Dahal</v>
-      </c>
-      <c r="B8" t="str">
-        <v>083MSNCS07</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Malware Classification Using Deep Learning Techniques</v>
-      </c>
-      <c r="D8" t="str">
-        <v>083</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Cluster 1</v>
-      </c>
-      <c r="F8" t="str">
-        <v>MSc in Network and Cyber Security</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Dr. Nilima Joshi</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Dr. Prajwal Ghimire</v>
-      </c>
-      <c r="I8" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Uma Lama</v>
-      </c>
-      <c r="B9" t="str">
-        <v>083MSNCS08</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Digital Forensics Investigation Framework for Nepali Organizations</v>
-      </c>
-      <c r="D9" t="str">
-        <v>083</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Cluster 1</v>
-      </c>
-      <c r="F9" t="str">
-        <v>MSc in Network and Cyber Security</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Prof. Dr. Raju Poudel</v>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
         <v>Assoc. Prof. Dr. Manisha Aryal</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>